<commit_message>
adequando teste1 a nova arquitetura
</commit_message>
<xml_diff>
--- a/consolidated_data.xlsx
+++ b/consolidated_data.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="consolidated_data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -592,67 +592,99 @@
       <c r="B2" t="n">
         <v>11.42878913879395</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v/>
+      </c>
       <c r="D2" t="n">
         <v>13.06970024108887</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v/>
+      </c>
       <c r="F2" t="n">
         <v>26.01000022888184</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v/>
+      </c>
       <c r="H2" t="n">
         <v>17.52531242370605</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v/>
+      </c>
       <c r="J2" t="n">
         <v>13.94576263427734</v>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v/>
+      </c>
       <c r="L2" t="n">
         <v>8.269610404968262</v>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v/>
+      </c>
       <c r="N2" t="n">
         <v>4.190000057220459</v>
       </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v/>
+      </c>
       <c r="P2" t="n">
         <v>29.39991760253906</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="Q2" t="n">
+        <v/>
+      </c>
       <c r="R2" t="n">
         <v>27.68414878845215</v>
       </c>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v/>
+      </c>
       <c r="T2" t="n">
         <v>45.34999847412109</v>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v/>
+      </c>
       <c r="V2" t="n">
         <v>21.22658348083496</v>
       </c>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v/>
+      </c>
       <c r="X2" t="n">
         <v>24.36904144287109</v>
       </c>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" t="n">
+        <v/>
+      </c>
       <c r="Z2" t="n">
         <v>55.34389495849609</v>
       </c>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="n">
+        <v/>
+      </c>
       <c r="AB2" t="n">
         <v>66.19867706298828</v>
       </c>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AC2" t="n">
+        <v/>
+      </c>
       <c r="AD2" t="n">
         <v>62.3103141784668</v>
       </c>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AE2" t="n">
+        <v/>
+      </c>
       <c r="AF2" t="n">
         <v>33.9872932434082</v>
       </c>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10045,8 +10077,12 @@
       <c r="E94" t="n">
         <v>0.002700380281896564</v>
       </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
+      <c r="F94" t="n">
+        <v/>
+      </c>
+      <c r="G94" t="n">
+        <v/>
+      </c>
       <c r="H94" t="n">
         <v>12.77536106109619</v>
       </c>
@@ -10147,7 +10183,9 @@
       <c r="F95" t="n">
         <v>27.79999923706055</v>
       </c>
-      <c r="G95" t="inlineStr"/>
+      <c r="G95" t="n">
+        <v/>
+      </c>
       <c r="H95" t="n">
         <v>12.71824264526367</v>
       </c>

</xml_diff>